<commit_message>
Sync roadmap from Nextcloud
</commit_message>
<xml_diff>
--- a/data/durf-roadmap.xlsx
+++ b/data/durf-roadmap.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="218">
   <si>
     <t xml:space="preserve">DURF roadmap — how to edit this workbook</t>
   </si>
@@ -412,10 +412,34 @@
     <t xml:space="preserve">1 Digital sovereignty health CRIS/Repo Dashboard: chart with ratio of metadata records containing a link to a file (PDF) on the institutional domain, per repo over time.</t>
   </si>
   <si>
-    <t xml:space="preserve">2, 4, 6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. aanvullen van datapunten UKBsis formate,OA. Pascal schrijf dit verder uit. Welke tussenstapjes.</t>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Write a proposal (2)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Approval of the proposal (3)
+Collect data for the monitor (4)
+Develop the monitor (4 – 5)
+Launch of the monitor (6)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Started</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- data delivery (all insitutions)
+- development of the monitor (WUR?)</t>
   </si>
   <si>
     <t xml:space="preserve">Create inventory of existing tools and methods for full-text capture</t>
@@ -693,7 +717,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="&quot;€ &quot;#,##0"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -745,6 +769,11 @@
       <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <i val="true"/>
@@ -854,7 +883,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -919,11 +948,15 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1641,7 +1674,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="25.95"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="46"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="38"/>
@@ -2103,7 +2136,7 @@
       <c r="K15" s="8"/>
       <c r="L15" s="8"/>
     </row>
-    <row r="16" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="15">
         <v>3</v>
       </c>
@@ -2122,19 +2155,19 @@
       <c r="F16" s="15">
         <v>6</v>
       </c>
-      <c r="G16" s="15" t="s">
+      <c r="G16" s="16" t="s">
         <v>126</v>
       </c>
       <c r="H16" s="8" t="s">
         <v>113</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="J16" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="K16" s="8"/>
+      <c r="J16" s="8"/>
+      <c r="K16" s="8" t="s">
+        <v>128</v>
+      </c>
       <c r="L16" s="8"/>
     </row>
     <row r="17" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2142,10 +2175,10 @@
         <v>3</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D17" s="8" t="s">
         <v>78</v>
@@ -2170,13 +2203,13 @@
         <v>3</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E18" s="15">
         <v>12</v>
@@ -2198,13 +2231,13 @@
         <v>3</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E19" s="15">
         <v>24</v>
@@ -2226,13 +2259,13 @@
         <v>4</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E20" s="15">
         <v>3</v>
@@ -2254,13 +2287,13 @@
         <v>4</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E21" s="15">
         <v>12</v>
@@ -2282,10 +2315,10 @@
         <v>4</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D22" s="8" t="s">
         <v>120</v>
@@ -2312,13 +2345,13 @@
         <v>4</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E23" s="15">
         <v>12</v>
@@ -2340,10 +2373,10 @@
         <v>5</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D24" s="8" t="s">
         <v>78</v>
@@ -2356,7 +2389,7 @@
       </c>
       <c r="G24" s="15"/>
       <c r="H24" s="8" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="I24" s="7" t="s">
         <v>80</v>
@@ -2370,13 +2403,13 @@
         <v>5</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E25" s="15">
         <v>6</v>
@@ -2398,10 +2431,10 @@
         <v>5</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D26" s="8" t="s">
         <v>120</v>
@@ -2414,7 +2447,7 @@
       </c>
       <c r="G26" s="15"/>
       <c r="H26" s="8" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="I26" s="7" t="s">
         <v>80</v>
@@ -2428,10 +2461,10 @@
         <v>6</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D27" s="8" t="s">
         <v>83</v>
@@ -2443,14 +2476,14 @@
         <v>25</v>
       </c>
       <c r="G27" s="15" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H27" s="8"/>
       <c r="I27" s="7" t="s">
         <v>80</v>
       </c>
       <c r="J27" s="8" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="K27" s="8"/>
       <c r="L27" s="8"/>
@@ -2460,10 +2493,10 @@
         <v>6</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D28" s="8" t="s">
         <v>78</v>
@@ -2475,14 +2508,14 @@
         <v>42</v>
       </c>
       <c r="G28" s="15" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H28" s="8"/>
       <c r="I28" s="7" t="s">
         <v>80</v>
       </c>
       <c r="J28" s="8" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="K28" s="8"/>
       <c r="L28" s="8"/>
@@ -2492,10 +2525,10 @@
         <v>6</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D29" s="8" t="s">
         <v>78</v>
@@ -2507,14 +2540,14 @@
         <v>45</v>
       </c>
       <c r="G29" s="15" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="H29" s="8"/>
       <c r="I29" s="7" t="s">
         <v>80</v>
       </c>
       <c r="J29" s="8" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="K29" s="8"/>
       <c r="L29" s="8"/>
@@ -2524,10 +2557,10 @@
         <v>6</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D30" s="8" t="s">
         <v>120</v>
@@ -2546,7 +2579,7 @@
         <v>80</v>
       </c>
       <c r="J30" s="8" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K30" s="8"/>
       <c r="L30" s="8"/>
@@ -2556,10 +2589,10 @@
         <v>6</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D31" s="8" t="s">
         <v>109</v>
@@ -2571,7 +2604,7 @@
         <v>9</v>
       </c>
       <c r="G31" s="15" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="H31" s="8"/>
       <c r="I31" s="7" t="s">
@@ -2628,16 +2661,16 @@
         <v>24</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2645,16 +2678,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>177</v>
-      </c>
-      <c r="D2" s="16">
+        <v>178</v>
+      </c>
+      <c r="D2" s="17">
         <v>92000</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2662,16 +2695,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>180</v>
-      </c>
-      <c r="D3" s="16">
+        <v>181</v>
+      </c>
+      <c r="D3" s="17">
         <v>3000</v>
       </c>
       <c r="E3" s="15" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2679,16 +2712,16 @@
         <v>2</v>
       </c>
       <c r="B4" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="D4" s="17">
+        <v>20000</v>
+      </c>
+      <c r="E4" s="15" t="s">
         <v>182</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="D4" s="16">
-        <v>20000</v>
-      </c>
-      <c r="E4" s="15" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2696,16 +2729,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>185</v>
-      </c>
-      <c r="D5" s="16">
+        <v>186</v>
+      </c>
+      <c r="D5" s="17">
         <v>40000</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2713,16 +2746,16 @@
         <v>2</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>180</v>
-      </c>
-      <c r="D6" s="16">
+        <v>181</v>
+      </c>
+      <c r="D6" s="17">
         <v>3000</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2730,16 +2763,16 @@
         <v>2</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>187</v>
-      </c>
-      <c r="D7" s="16">
+        <v>188</v>
+      </c>
+      <c r="D7" s="17">
         <v>27000</v>
       </c>
       <c r="E7" s="15" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2747,16 +2780,16 @@
         <v>2</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>188</v>
-      </c>
-      <c r="D8" s="16">
+        <v>189</v>
+      </c>
+      <c r="D8" s="17">
         <v>21000</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2764,16 +2797,16 @@
         <v>3</v>
       </c>
       <c r="B9" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="D9" s="17">
+        <v>20000</v>
+      </c>
+      <c r="E9" s="15" t="s">
         <v>182</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="D9" s="16">
-        <v>20000</v>
-      </c>
-      <c r="E9" s="15" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2781,16 +2814,16 @@
         <v>3</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>185</v>
-      </c>
-      <c r="D10" s="16">
+        <v>186</v>
+      </c>
+      <c r="D10" s="17">
         <v>40000</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2798,16 +2831,16 @@
         <v>3</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>187</v>
-      </c>
-      <c r="D11" s="16">
+        <v>188</v>
+      </c>
+      <c r="D11" s="17">
         <v>27000</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2815,16 +2848,16 @@
         <v>3</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>188</v>
-      </c>
-      <c r="D12" s="16">
+        <v>189</v>
+      </c>
+      <c r="D12" s="17">
         <v>21000</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2832,16 +2865,16 @@
         <v>4</v>
       </c>
       <c r="B13" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="D13" s="17">
+        <v>20000</v>
+      </c>
+      <c r="E13" s="15" t="s">
         <v>182</v>
-      </c>
-      <c r="C13" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="D13" s="16">
-        <v>20000</v>
-      </c>
-      <c r="E13" s="15" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2849,16 +2882,16 @@
         <v>4</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>185</v>
-      </c>
-      <c r="D14" s="16">
+        <v>186</v>
+      </c>
+      <c r="D14" s="17">
         <v>40000</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2866,16 +2899,16 @@
         <v>4</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>188</v>
-      </c>
-      <c r="D15" s="16">
+        <v>189</v>
+      </c>
+      <c r="D15" s="17">
         <v>21000</v>
       </c>
       <c r="E15" s="15" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2883,16 +2916,16 @@
         <v>5</v>
       </c>
       <c r="B16" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="D16" s="17">
+        <v>20000</v>
+      </c>
+      <c r="E16" s="15" t="s">
         <v>182</v>
-      </c>
-      <c r="C16" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="D16" s="16">
-        <v>20000</v>
-      </c>
-      <c r="E16" s="15" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2900,16 +2933,16 @@
         <v>5</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>185</v>
-      </c>
-      <c r="D17" s="16">
+        <v>186</v>
+      </c>
+      <c r="D17" s="17">
         <v>40000</v>
       </c>
       <c r="E17" s="15" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2917,16 +2950,16 @@
         <v>6</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>189</v>
-      </c>
-      <c r="D18" s="16">
+        <v>190</v>
+      </c>
+      <c r="D18" s="17">
         <v>50000</v>
       </c>
       <c r="E18" s="15" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
   </sheetData>
@@ -2966,7 +2999,7 @@
         <v>24</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>71</v>
@@ -2977,10 +3010,10 @@
         <v>5</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2988,10 +3021,10 @@
         <v>5</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2999,10 +3032,10 @@
         <v>5</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
   </sheetData>
@@ -3033,79 +3066,79 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>201</v>
-      </c>
-      <c r="C2" s="17" t="s">
         <v>202</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>203</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>204</v>
-      </c>
-      <c r="C3" s="17" t="s">
         <v>205</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>207</v>
-      </c>
-      <c r="C4" s="17" t="s">
         <v>208</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B5" s="8">
         <v>48</v>
       </c>
-      <c r="C5" s="17" t="s">
-        <v>210</v>
+      <c r="C5" s="18" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="C6" s="17" t="s">
         <v>213</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>215</v>
-      </c>
-      <c r="C7" s="17" t="s">
         <v>216</v>
+      </c>
+      <c r="C7" s="18" t="s">
+        <v>217</v>
       </c>
     </row>
   </sheetData>

</xml_diff>